<commit_message>
deocde: rs_decode mask, control_unit rev 2, regfile bypass
</commit_message>
<xml_diff>
--- a/supplemental/signal_origination.xlsx
+++ b/supplemental/signal_origination.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\riscv-power-aware\supplemental\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F7F0B89F-BF02-4B35-94E6-7A38C7FA0B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F070F32-267B-412D-AE59-1B17720093B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="11260" xr2:uid="{614D22FF-3AA2-4042-A943-E9B88D054E6A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{614D22FF-3AA2-4042-A943-E9B88D054E6A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>IBUS</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Fetch</t>
   </si>
@@ -63,6 +60,39 @@
   </si>
   <si>
     <t>Flush</t>
+  </si>
+  <si>
+    <t>INSTR</t>
+  </si>
+  <si>
+    <t>PCSEL</t>
+  </si>
+  <si>
+    <t>NEXT_PC</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>PC_PLUS4</t>
+  </si>
+  <si>
+    <t>PREDICT</t>
+  </si>
+  <si>
+    <t>FETCH_TARGET</t>
+  </si>
+  <si>
+    <t>TARGET_VALID</t>
+  </si>
+  <si>
+    <t>IS_JAL</t>
+  </si>
+  <si>
+    <t>PREDICT_TAKEN</t>
+  </si>
+  <si>
+    <t>LOAD_IF</t>
   </si>
 </sst>
 </file>
@@ -434,39 +464,92 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F5CB88C-A596-49C8-997B-93FB27E03DD4}">
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="5" width="14.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C4" t="s">
-        <v>7</v>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated decode to include the forwarding mux and unit to resolve forwarding slection a stage earlier
</commit_message>
<xml_diff>
--- a/supplemental/signal_origination.xlsx
+++ b/supplemental/signal_origination.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\riscv-power-aware\supplemental\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F070F32-267B-412D-AE59-1B17720093B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7D9DFA-327A-4207-B4B0-874570000316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{614D22FF-3AA2-4042-A943-E9B88D054E6A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{614D22FF-3AA2-4042-A943-E9B88D054E6A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Fetch</t>
   </si>
@@ -56,12 +56,6 @@
     <t>WB</t>
   </si>
   <si>
-    <t>Branch</t>
-  </si>
-  <si>
-    <t>Flush</t>
-  </si>
-  <si>
     <t>INSTR</t>
   </si>
   <si>
@@ -93,14 +87,88 @@
   </si>
   <si>
     <t>LOAD_IF</t>
+  </si>
+  <si>
+    <t>RS1</t>
+  </si>
+  <si>
+    <t>RS2</t>
+  </si>
+  <si>
+    <t>RD</t>
+  </si>
+  <si>
+    <t>FUNCT3</t>
+  </si>
+  <si>
+    <t>IMMSRC</t>
+  </si>
+  <si>
+    <t>IMM_EXT</t>
+  </si>
+  <si>
+    <t>RD1</t>
+  </si>
+  <si>
+    <t>RD2</t>
+  </si>
+  <si>
+    <t>SRC1SEL</t>
+  </si>
+  <si>
+    <t>SRC2SEL</t>
+  </si>
+  <si>
+    <t>OP_A</t>
+  </si>
+  <si>
+    <t>OP_B</t>
+  </si>
+  <si>
+    <t>ALUSEL</t>
+  </si>
+  <si>
+    <t>WD4SEL</t>
+  </si>
+  <si>
+    <t>BRANCH</t>
+  </si>
+  <si>
+    <t>IS_JALR</t>
+  </si>
+  <si>
+    <t>MEMRD</t>
+  </si>
+  <si>
+    <t>MEMWR</t>
+  </si>
+  <si>
+    <t>REGWR</t>
+  </si>
+  <si>
+    <t>STALL</t>
+  </si>
+  <si>
+    <t>BUBBLE</t>
+  </si>
+  <si>
+    <t>REDIRECT_EN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -128,8 +196,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,92 +533,192 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F5CB88C-A596-49C8-997B-93FB27E03DD4}">
-  <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E34"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="5" width="14.7109375" customWidth="1"/>
+    <col min="1" max="5" width="14.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B28" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B29" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B30" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B32" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C34" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Verified proper branch prediction and forwarding and stalling
</commit_message>
<xml_diff>
--- a/supplemental/signal_origination.xlsx
+++ b/supplemental/signal_origination.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\riscv-power-aware\supplemental\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF2ECDE0-3EBB-4C40-9988-DC40B66550E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8922470F-E780-47AA-AB9A-7942EE352126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{614D22FF-3AA2-4042-A943-E9B88D054E6A}"/>
   </bookViews>
@@ -437,36 +437,6 @@
     <t>WB_VALUE[31..0]</t>
   </si>
   <si>
-    <t>Branch/JAL target, computed in IF by branch_target_calc from the IF instruction and PC. Only meaningful when TARGET_VALID=1 — junk otherwise, so don't read it on non-branches. Feeds PCMUX.D1 in IF and REDIRECT_MUX.D1 in EX (the address used when a taken branch was mispredicted). Computing it in IF is what makes a correct prediction cost 0 cycles.</t>
-  </si>
-  <si>
-    <t>Program counter of the instruction in this stage. ID_EX_PC is the BHT's training index, so it must be the EX instruction's PC — if it were fetch's PC the predictor would train the wrong counter silently. There is no PC output pin: read PC_PLUS4 minus 4.</t>
-  </si>
-  <si>
-    <t>PC+4 from the IF adder. Serves as PCMUX.D0 (sequential fetch) and, in EX, as the link value for JAL/JALR and as the redirect address when a predicted-taken branch resolves not-taken.</t>
-  </si>
-  <si>
-    <t>Records that fetch actually redirected to this instruction's target. pc_sel_logic sets it only when PCSEL=001, and clears it on RST, REDIRECT_EN and STALL. Compared against BR_TAKEN in EX to detect a mispredict. If this is stuck at 0 the core still runs correctly but every taken branch reports a mispredict and the predictor buys nothing.</t>
-  </si>
-  <si>
-    <t>Raw instruction word out of the IROM (unregistered M9K output). IF_ID_INSTR is the copy decode actually works on. The IBUS pin taps the IF copy, so on a waveform it runs ONE INSTRUCTION AHEAD of what ID is decoding.</t>
-  </si>
-  <si>
-    <t>branch_target_calc decoded opcode 1101111. Forces TAKE_TARGET in pc_sel_logic — a JAL is unconditionally taken, so no prediction is consulted.</t>
-  </si>
-  <si>
-    <t>(NOT STALL) OR RST. Enables PC_REG, the IROM read (rden), and all five IF/ID registers. Goes low for exactly one cycle per load-use stall — that low pulse IS the front end holding still.</t>
-  </si>
-  <si>
-    <t>PCMUX output. Latched by PC_REG and the IROM address register on the same edge, which is what keeps PC and INSTR aligned. Only bits [11..2] reach the IROM address port.</t>
-  </si>
-  <si>
-    <t>PCMUX select from pc_sel_logic. 000 = PC+4, 001 = branch target, 010 = redirect, 011 = reset zero, 100 = hold. Priority RST &gt; REDIRECT_EN &gt; STALL &gt; predicted-taken &gt; sequential. Reads 100 only during a stall; if it never does, the hold arm is not wired.</t>
-  </si>
-  <si>
-    <t>BHT saturating-counter output for this PC. Watch it settle: a loop branch should reach 1 after one or two iterations and stay there. If it oscillates, the training index or UPDATE_EN is wrong.</t>
-  </si>
-  <si>
     <t>branch_target_calc says the target is computable in IF — B-type or JAL. Low for JALR (target needs a register value) and for every non-control instruction.</t>
   </si>
   <si>
@@ -545,52 +515,82 @@
     <t>OPAMUX select. 1 = PC (AUIPC, JAL), 0 = register rs1.</t>
   </si>
   <si>
-    <t>OPBMUX select. 1 = immediate, 0 = register rs2. Also tells forwarding_unit to suppress B-side forwarding, since an immediate has no producer.</t>
-  </si>
-  <si>
-    <t>Load-use hazard: a load is in EX and the instruction in ID reads its destination register. Holds PC_REG, the IROM and IF/ID while bubbling ID/EX. Exactly one cycle per hazard. No STALL pin exists — read the FLUSH pin in a program with no branches.</t>
-  </si>
-  <si>
-    <t>rs_decode says this opcode genuinely reads rs1. Masks the register file's read DATA to zero rather than masking the address, so the 32:1 read can start straight off the IROM. It OUTRANKS the write-first bypass — that ordering is load-bearing.</t>
-  </si>
-  <si>
     <t>Same as USE_A1, for rs2.</t>
   </si>
   <si>
-    <t>ALU result or PC+4, already selected by WBVAL_MUX in EX. Collapsing the choice here is why writeback is a 2:1 instead of a 4:1, and why JAL's link value forwards correctly.</t>
-  </si>
-  <si>
-    <t>Marks the slot as holding a real instruction rather than a bubble. Currently tied to VCC at ID/EX, so it reads 1 even for the SECOND bubble after a mispredict — add an IFID_VALID register before trusting it for retire counts or pipeline utilisation.</t>
-  </si>
-  <si>
-    <t>Raw ALU output. Also the load/store address: it crosses into the memory block combinationally as A_EX, so the M9K's own address register is the EX/MEM boundary for the data path.</t>
-  </si>
-  <si>
-    <t>(BR_TAKEN XOR ID_EX_PREDICT_TAKEN) AND ID_EX_BRANCH. High for exactly one cycle, the cycle the branch sits in EX. A correctly predicted branch must NOT raise this — that is the real test of the predictor.</t>
-  </si>
-  <si>
-    <t>The XOR before the BRANCH gate. Goes high on any instruction whose BR_TAKEN and PREDICT_TAKEN happen to disagree, including non-branches. Ignore it unless ID_EX_BRANCH is also high.</t>
-  </si>
-  <si>
-    <t>MISPREDICT OR ID_EX_IS_JALR. The root flush signal, and the widest-fanout control signal in the core: it clears IF/ID directly, feeds the OR gate that makes BUBBLE (clearing ID/EX), and steers PCMUX to REDIRECT_PC. One cycle per mispredict.</t>
-  </si>
-  <si>
-    <t>REDIRECT_MUX output — the corrected fetch address. Selected by {ID_EX_IS_JALR, BR_TAKEN}: 00 = PC+4 (predicted taken, resolved not taken), 01 = branch target, 1x = JALR target from the ALU with bit 0 forced to zero.</t>
-  </si>
-  <si>
-    <t>BR_TAKEN routed back to the BHT as the actual outcome. Paired with ID_EX_PC (the index) and ID_EX_BRANCH (the update enable). If this never toggles the predictor never learns.</t>
-  </si>
-  <si>
-    <t>Hard-wired 0, concatenated with ALU_F[31:1] to clear bit 0 of a JALR target as RV32I requires.</t>
-  </si>
-  <si>
-    <t>DMEM read data, already width-adjusted and sign/zero-extended per FUNCT3. Forwarded to decode from HERE (the MEM stage), not from MEM_WB_RDM — the producer and the consumer are the same instruction one stage apart.</t>
-  </si>
-  <si>
-    <t>Final writeback data: MEM_WB_RDM on a load, MEM_WB_WB_VALUE otherwise, selected by MEM_WB_MEMRD. This is the WD3 pin — the most useful single signal for checking a program executed correctly.</t>
-  </si>
-  <si>
     <t>What it is/What it does</t>
+  </si>
+  <si>
+    <t>Program counter of the instruction in this stage. ID_EX_PC is the BHT's training index, so it must be the EX instruction's PC.</t>
+  </si>
+  <si>
+    <t>Branch/JAL target, computed in IF by branch_target_calc from the IF instruction and PC. Only meaningful when TARGET_VALID=1 — junk otherwise. Feeds PCMUX in IF and REDIRECT_MUX in EX. Computing it in IF makes correct predictions have zero cost.</t>
+  </si>
+  <si>
+    <t>PC+4 from the IF adder. Serves as PCMUX and, in EX, as the link value for JAL/JALR and as the redirect address when a predicted-taken branch resolves not-taken.</t>
+  </si>
+  <si>
+    <t>Records that fetch actually redirected to this instruction's target. pc_sel_logic sets it only when PCSEL=001. Clears is on RST, REDIRECt_EN, and STALL. Compared against BR_TAKEN in EX to detect a mispredict.</t>
+  </si>
+  <si>
+    <t>Raw instruction word out of the IROM. IF_ID_INSTR is the copy decode actually works on. The IBUS pin taps the IF version.</t>
+  </si>
+  <si>
+    <t>Final writeback data</t>
+  </si>
+  <si>
+    <t>DMEM read data, already width-adjusted and sign/zero-extended per FUNCT3</t>
+  </si>
+  <si>
+    <t>Hard-wired 0, concatenated with ALU_F[31:1] to clear bit 0 of a JALR target</t>
+  </si>
+  <si>
+    <t>BR_TAKEN routed back to the BHT as the actual outcome. Paired with ID_EX_PC and ID_EX_BRANCH. If this never toggles the predictor never learns.</t>
+  </si>
+  <si>
+    <t>REDIRECT_MUX output — the corrected fetch address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISPREDICT OR ID_EX_IS_JALR. The root flush signal, and the widest-fanout control signal in the core: it clears IF/ID directly, feeds the OR gate that makes BUBBLE </t>
+  </si>
+  <si>
+    <t>The XOR before the BRANCH gate. Goes high on any instruction whose BR_TAKEN and PREDICT_TAKEN happen to disagree</t>
+  </si>
+  <si>
+    <t>(BR_TAKEN XOR ID_EX_PREDICT_TAKEN) AND ID_EX_BRANCH</t>
+  </si>
+  <si>
+    <t>Raw ALU output. Also the load/store address</t>
+  </si>
+  <si>
+    <t>Marks the slot as holding a real instruction rather than a bubble</t>
+  </si>
+  <si>
+    <t>ALU result or PC+4, already selected by WBVAL_MUX in EX</t>
+  </si>
+  <si>
+    <t>rs_decodesays opcode reads rs1. Masks the register file's read DATA to zero rather than masking the address</t>
+  </si>
+  <si>
+    <t>Load-use hazard:</t>
+  </si>
+  <si>
+    <t>OPBMUX select. 1 = immediate, 0 = register rs2. Also tells forwarding_unit to suppress B-side forwarding</t>
+  </si>
+  <si>
+    <t>branch_target_calc decoded opcode 1101111. JAL is unconditional</t>
+  </si>
+  <si>
+    <t>(NOT STALL) OR RST. Enables PC_REG, the IROM read (rden), and all five IF/ID registers. Goes low for exactly one cycle per load-use stall</t>
+  </si>
+  <si>
+    <t>PCMUX output. Latched by PC_REG and the IROM address register on the same edge. bits [11..2] reach the IROM address port.</t>
+  </si>
+  <si>
+    <t>PCMUX select from pc_sel_logic. 000 = PC+4, 001 = branch target, 010 = redirect, 011 = reset zero, 100 = hold.</t>
+  </si>
+  <si>
+    <t>BHT saturating-counter output for this PC</t>
   </si>
 </sst>
 </file>
@@ -1012,10 +1012,10 @@
         <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -1035,10 +1035,10 @@
         <v>75</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1058,10 +1058,10 @@
         <v>77</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1081,10 +1081,10 @@
         <v>79</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1104,10 +1104,10 @@
         <v>80</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1124,10 +1124,10 @@
         <v>81</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1141,10 +1141,10 @@
         <v>12</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -1158,7 +1158,7 @@
         <v>14</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>138</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1175,10 +1175,10 @@
         <v>82</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -1192,10 +1192,10 @@
         <v>83</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1209,7 +1209,7 @@
         <v>10</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>141</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1226,7 +1226,7 @@
         <v>11</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -1252,7 +1252,7 @@
         <v>86</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -1278,7 +1278,7 @@
         <v>90</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -1304,7 +1304,7 @@
         <v>93</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1327,7 +1327,7 @@
         <v>96</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1350,7 +1350,7 @@
         <v>98</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1373,7 +1373,7 @@
         <v>100</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -1393,7 +1393,7 @@
         <v>102</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -1413,7 +1413,7 @@
         <v>103</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1433,7 +1433,7 @@
         <v>104</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1453,7 +1453,7 @@
         <v>105</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1473,7 +1473,7 @@
         <v>106</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -1493,7 +1493,7 @@
         <v>108</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -1510,7 +1510,7 @@
         <v>109</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1527,7 +1527,7 @@
         <v>110</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1544,7 +1544,7 @@
         <v>111</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -1561,7 +1561,7 @@
         <v>33</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
@@ -1578,7 +1578,7 @@
         <v>112</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1595,7 +1595,7 @@
         <v>113</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
@@ -1612,7 +1612,7 @@
         <v>114</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
@@ -1629,7 +1629,7 @@
         <v>115</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1646,7 +1646,7 @@
         <v>116</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
@@ -1663,7 +1663,7 @@
         <v>117</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -1680,7 +1680,7 @@
         <v>118</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
@@ -1697,7 +1697,7 @@
         <v>119</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
@@ -1714,7 +1714,7 @@
         <v>21</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -1731,10 +1731,10 @@
         <v>22</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -1748,10 +1748,10 @@
         <v>32</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>49</v>
       </c>
@@ -1765,7 +1765,7 @@
         <v>49</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
@@ -1782,10 +1782,10 @@
         <v>50</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>51</v>
       </c>
@@ -1805,10 +1805,10 @@
         <v>122</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>52</v>
       </c>
@@ -1828,10 +1828,10 @@
         <v>125</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>53</v>
       </c>
@@ -1848,10 +1848,10 @@
         <v>127</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>54</v>
       </c>
@@ -1865,10 +1865,10 @@
         <v>54</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>55</v>
       </c>
@@ -1882,10 +1882,10 @@
         <v>55</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>34</v>
       </c>
@@ -1899,10 +1899,10 @@
         <v>34</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>56</v>
       </c>
@@ -1916,10 +1916,10 @@
         <v>128</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>57</v>
       </c>
@@ -1933,10 +1933,10 @@
         <v>57</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>58</v>
       </c>
@@ -1950,10 +1950,10 @@
         <v>58</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>59</v>
       </c>
@@ -1970,10 +1970,10 @@
         <v>130</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>60</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>131</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>182</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>